<commit_message>
Textile workshop quote: 15 seats, Laura 13k/h, paint kits, restaurant budget 500k (editable), spare kimono
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FV7y6XEE3x9ogCMyfe3pnd
</commit_message>
<xml_diff>
--- a/docs/sesion-2026-10-02/cotizacion-taller-pintura-textil.xlsx
+++ b/docs/sesion-2026-10-02/cotizacion-taller-pintura-textil.xlsx
@@ -218,7 +218,7 @@
   <commentList>
     <comment ref="B6" authorId="0" shapeId="0">
       <text>
-        <t>ESTIMADO. Con tres acompañantes caben unas 10–12 personas.</t>
+        <t>Dato de Sara: 15 cupos.</t>
       </text>
     </comment>
     <comment ref="B7" authorId="0" shapeId="0">
@@ -238,72 +238,87 @@
     </comment>
     <comment ref="B12" authorId="0" shapeId="0">
       <text>
-        <t>ESTIMADO. Es el costo MÁS importante: pon el costo real de producción de un kimono de Alado.</t>
+        <t>ESTIMADO Y PENDIENTE: Sara no alcanzó a enviar el costo real. Es el costo más importante.</t>
       </text>
     </comment>
     <comment ref="B13" authorId="0" shapeId="0">
       <text>
+        <t>Recomendado: 1 por cada 15 personas. Pon 0 si no quieres repuestos.</t>
+      </text>
+    </comment>
+    <comment ref="B14" authorId="0" shapeId="0">
+      <text>
+        <t>Dato de Sara: Mercado Libre.</t>
+      </text>
+    </comment>
+    <comment ref="B15" authorId="0" shapeId="0">
+      <text>
+        <t>Dato de Sara: 1 kit cada 3 personas.</t>
+      </text>
+    </comment>
+    <comment ref="B16" authorId="0" shapeId="0">
+      <text>
+        <t>ESTIMADO. Si usan retazos de Alado, puede ser $0.</t>
+      </text>
+    </comment>
+    <comment ref="B17" authorId="0" shapeId="0">
+      <text>
         <t>ESTIMADO.</t>
       </text>
     </comment>
-    <comment ref="B14" authorId="0" shapeId="0">
+    <comment ref="B18" authorId="0" shapeId="0">
+      <text>
+        <t>ESTIMADO. Pon $0 si lo pone el restaurante.</t>
+      </text>
+    </comment>
+    <comment ref="B19" authorId="0" shapeId="0">
       <text>
         <t>ESTIMADO.</t>
       </text>
     </comment>
-    <comment ref="B15" authorId="0" shapeId="0">
-      <text>
-        <t>ESTIMADO. Pon $0 si lo pone un aliado.</t>
-      </text>
-    </comment>
-    <comment ref="B16" authorId="0" shapeId="0">
+    <comment ref="B20" authorId="0" shapeId="0">
+      <text>
+        <t>Las 4 horas son dato de Sara; la hora de preparación es estimada.</t>
+      </text>
+    </comment>
+    <comment ref="B21" authorId="0" shapeId="0">
+      <text>
+        <t>Dato de Sara.</t>
+      </text>
+    </comment>
+    <comment ref="B22" authorId="0" shapeId="0">
+      <text>
+        <t>Son los fundadores. Pon un valor si quieres imputar su tiempo.</t>
+      </text>
+    </comment>
+    <comment ref="B23" authorId="0" shapeId="0">
+      <text>
+        <t>ESTIMADO. Se compran una vez; en el próximo taller cuestan menos.</t>
+      </text>
+    </comment>
+    <comment ref="B24" authorId="0" shapeId="0">
+      <text>
+        <t>Los del taller de cerámica se pueden reutilizar.</t>
+      </text>
+    </comment>
+    <comment ref="B25" authorId="0" shapeId="0">
       <text>
         <t>ESTIMADO.</t>
       </text>
     </comment>
-    <comment ref="B17" authorId="0" shapeId="0">
-      <text>
-        <t>Las 4 horas son dato de Sara; la hora de preparación es estimada.</t>
-      </text>
-    </comment>
-    <comment ref="B18" authorId="0" shapeId="0">
-      <text>
-        <t>ESTIMADO: usé la tarifa de Lizeth. Cámbiala por la de Laura.</t>
-      </text>
-    </comment>
-    <comment ref="B19" authorId="0" shapeId="0">
-      <text>
-        <t>Son los fundadores. Pon un valor si quieres imputar su tiempo.</t>
-      </text>
-    </comment>
-    <comment ref="B20" authorId="0" shapeId="0">
-      <text>
-        <t>ESTIMADO. Se compran una vez; en el próximo taller cuestan menos.</t>
-      </text>
-    </comment>
-    <comment ref="B21" authorId="0" shapeId="0">
-      <text>
-        <t>Los del taller de cerámica se pueden reutilizar.</t>
-      </text>
-    </comment>
-    <comment ref="B22" authorId="0" shapeId="0">
-      <text>
-        <t>ESTIMADO.</t>
-      </text>
-    </comment>
-    <comment ref="B23" authorId="0" shapeId="0">
-      <text>
-        <t>Pon aquí el valor del contenido si se carga a este taller.</t>
-      </text>
-    </comment>
-    <comment ref="B44" authorId="0" shapeId="0">
+    <comment ref="B26" authorId="0" shapeId="0">
+      <text>
+        <t>Sara indicó que el contenido lo dan Alejo, Laura y Andrés: $0. Pon un valor si se carga contenido de redes a este taller.</t>
+      </text>
+    </comment>
+    <comment ref="B49" authorId="0" shapeId="0">
       <text>
         <t>Propuesta de partida. Súbelo o bájalo según lo que negocies.</t>
       </text>
     </comment>
-    <comment ref="B47" authorId="0" shapeId="0">
-      <text>
-        <t>Escribe el valor acordado. La ganancia de abajo se recalcula sola.</t>
+    <comment ref="B52" authorId="0" shapeId="0">
+      <text>
+        <t>Presupuesto de Sara para el restaurante. Cámbialo cuando negocies: la ganancia se recalcula sola.</t>
       </text>
     </comment>
   </commentList>
@@ -599,10 +614,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G82"/>
+  <dimension ref="A1:G87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="66" customWidth="1" min="1" max="1"/>
+    <col width="68" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
@@ -621,7 +636,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>4 horas · con Andrés, Alejo y Laura · cada persona pinta y se lleva un kimono</t>
+          <t>4 horas · con Andrés, Alejo y Laura · en un restaurante · cada persona pinta y se lleva un kimono</t>
         </is>
       </c>
     </row>
@@ -646,7 +661,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7">
@@ -712,799 +727,851 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Pinturas textiles (por persona)</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="n">
-        <v>25000</v>
+          <t>Kimonos de repuesto por si alguno se daña (cantidad total)</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Pinceles y materiales de pintura que se gastan (por persona)</t>
+          <t>Kit de pintura textil · precio (6 frascos de 30 cc)</t>
         </is>
       </c>
       <c r="B14" s="6" t="n">
-        <v>8000</v>
+        <v>27600</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Refrigerio (por persona)</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="n">
-        <v>20000</v>
+          <t>Personas que comparten 1 kit</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Empaque para llevarse el kimono (por persona)</t>
+          <t>Hojas y retazos de tela para practicar (por persona)</t>
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>5000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Laura · horas (4 del taller + 1 de preparación)</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="n">
-        <v>5</v>
+          <t>Pinceles y materiales que se gastan (por persona)</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="n">
+        <v>8000</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Laura · valor por hora</t>
+          <t>Refrigerio (por persona)</t>
         </is>
       </c>
       <c r="B18" s="6" t="n">
-        <v>9000</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Andrés y Alejo (tiempo imputado, total)</t>
+          <t>Empaque para llevarse el kimono (por persona)</t>
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Pinceles, paletas y materiales reutilizables (total)</t>
-        </is>
-      </c>
-      <c r="B20" s="6" t="n">
-        <v>150000</v>
+          <t>Laura · horas (4 del taller + 1 de preparación)</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Delantales (total; $0 si ya los tienen)</t>
+          <t>Laura · valor por hora</t>
         </is>
       </c>
       <c r="B21" s="6" t="n">
-        <v>0</v>
+        <v>13000</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>Otros fijos: transporte, flores, promoción (total)</t>
+          <t>Andrés y Alejo (tiempo imputado, total)</t>
         </is>
       </c>
       <c r="B22" s="6" t="n">
-        <v>190000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Contenido del taller (piezas de Sara)</t>
+          <t>Materiales reutilizables: pinceles, paletas, vasos, cinta y plástico (total)</t>
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>0</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Pago al lugar o aliado (total) · se escribe en la sección «Pago al lugar»</t>
-        </is>
-      </c>
-      <c r="B24" s="8">
-        <f>B47</f>
-        <v/>
+          <t>Delantales (total; $0 si ya los tienen)</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Otros fijos: transporte, flores, promoción (total)</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="n">
+        <v>190000</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>RESULTADO</t>
-        </is>
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Contenido del taller (piezas de Sara)</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Kimonos pintados por persona</t>
-        </is>
-      </c>
-      <c r="B27" s="9">
-        <f>B11</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>Costo variable por persona (kimono, pinturas, materiales, refrigerio, empaque)</t>
-        </is>
-      </c>
-      <c r="B28" s="8">
-        <f>B11*B12+B13+B14+B15+B16</f>
+          <t>Pago al restaurante (total) · se escribe en la sección «Pago al restaurante»</t>
+        </is>
+      </c>
+      <c r="B27" s="8">
+        <f>B52</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>Costos fijos (Laura, fundadores, materiales, delantales, otros y contenido)</t>
-        </is>
-      </c>
-      <c r="B29" s="8">
-        <f>B17*B18+B19+B20+B21+B22+B23</f>
-        <v/>
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>RESULTADO</t>
+        </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>Costos base (fijos + variables × personas)</t>
-        </is>
-      </c>
-      <c r="B30" s="8">
-        <f>B29+B28*B6</f>
+          <t>Kits de pintura textil necesarios (redondeado hacia arriba)</t>
+        </is>
+      </c>
+      <c r="B30" s="9">
+        <f>ROUNDUP(B6/B15,0)</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>Imprevistos</t>
+          <t>Costo de la pintura textil</t>
         </is>
       </c>
       <c r="B31" s="8">
-        <f>B30*B10</f>
+        <f>B30*B14</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>Pago al lugar o aliado</t>
+          <t>Costo variable por persona (kimono, práctica, pinceles, refrigerio, empaque)</t>
         </is>
       </c>
       <c r="B32" s="8">
-        <f>B24</f>
+        <f>B11*B12+B16+B17+B18+B19</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="10" t="inlineStr">
-        <is>
-          <t>COSTO TOTAL del taller</t>
-        </is>
-      </c>
-      <c r="B33" s="11">
-        <f>B30+B31+B32</f>
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Kimonos de repuesto</t>
+        </is>
+      </c>
+      <c r="B33" s="8">
+        <f>B13*B12</f>
         <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>Costo por persona</t>
+          <t>Costos fijos (Laura, fundadores, materiales, delantales, otros, contenido y repuestos)</t>
         </is>
       </c>
       <c r="B34" s="8">
-        <f>B33/B6</f>
+        <f>B20*B21+B22+B23+B24+B25+B26+B33</f>
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>Ingresos por cupos (precio × personas)</t>
+          <t>Costos base (fijos + variables × personas + pintura)</t>
         </is>
       </c>
       <c r="B35" s="8">
-        <f>B7*B6</f>
+        <f>B34+B32*B6+B31</f>
         <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>Comisión de pago online</t>
+          <t>Imprevistos</t>
         </is>
       </c>
       <c r="B36" s="8">
-        <f>B35*B9</f>
+        <f>B35*B10</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="10" t="inlineStr">
-        <is>
-          <t>GANANCIA (después de pagarle al lugar)</t>
-        </is>
-      </c>
-      <c r="B37" s="11">
-        <f>B35-B36-B33</f>
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Pago al restaurante</t>
+        </is>
+      </c>
+      <c r="B37" s="8">
+        <f>B27</f>
         <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="10" t="inlineStr">
         <is>
-          <t>MARGEN real (ganancia ÷ ingresos)</t>
-        </is>
-      </c>
-      <c r="B38" s="12">
-        <f>IF(B35&gt;0,B37/B35,0)</f>
+          <t>COSTO TOTAL del taller</t>
+        </is>
+      </c>
+      <c r="B38" s="11">
+        <f>B35+B36+B37</f>
         <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>Ganancia por persona</t>
+          <t>Costo por persona</t>
         </is>
       </c>
       <c r="B39" s="8">
-        <f>B37/B6</f>
+        <f>B38/B6</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>¿Cumple el margen que quieres?</t>
-        </is>
-      </c>
-      <c r="B40" s="13">
-        <f>IF(B38&gt;=B8,"Sí, cumple","No: está por debajo")</f>
+          <t>Ingresos por cupos (precio × personas)</t>
+        </is>
+      </c>
+      <c r="B40" s="8">
+        <f>B7*B6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Comisión de pago online</t>
+        </is>
+      </c>
+      <c r="B41" s="8">
+        <f>B40*B9</f>
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="3" t="inlineStr">
-        <is>
-          <t>PAGO AL LUGAR O ALIADO (por ejemplo, un restaurante)</t>
-        </is>
+      <c r="A42" s="10" t="inlineStr">
+        <is>
+          <t>GANANCIA (después de pagarle al restaurante)</t>
+        </is>
+      </c>
+      <c r="B42" s="11">
+        <f>B40-B41-B38</f>
+        <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="4" t="inlineStr">
-        <is>
-          <t>Ganancia antes de pagarle al lugar</t>
-        </is>
-      </c>
-      <c r="B43" s="8">
-        <f>B35-B36-(B30+B31)</f>
+      <c r="A43" s="10" t="inlineStr">
+        <is>
+          <t>MARGEN real (ganancia ÷ ingresos)</t>
+        </is>
+      </c>
+      <c r="B43" s="12">
+        <f>IF(B40&gt;0,B42/B40,0)</f>
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>% de esa ganancia que le ofreces</t>
-        </is>
-      </c>
-      <c r="B44" s="7" t="n">
-        <v>0.3</v>
+          <t>Ganancia por persona</t>
+        </is>
+      </c>
+      <c r="B44" s="8">
+        <f>B42/B6</f>
+        <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="10" t="inlineStr">
-        <is>
-          <t>PAGO SUGERIDO (redondeado a $5.000)</t>
-        </is>
-      </c>
-      <c r="B45" s="11">
-        <f>MAX(0,ROUNDDOWN(B43*B44/5000,0)*5000)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
-        <is>
-          <t>…por persona</t>
-        </is>
-      </c>
-      <c r="B46" s="8">
-        <f>B45/B6</f>
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>¿Cumple el margen que quieres?</t>
+        </is>
+      </c>
+      <c r="B45" s="13">
+        <f>IF(B43&gt;=B8,"Sí, cumple","No: está por debajo")</f>
         <v/>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="10" t="inlineStr">
-        <is>
-          <t>LO QUE ACUERDAS PAGAR (escribe aquí; $0 si el lugar es de Alado)</t>
-        </is>
-      </c>
-      <c r="B47" s="6" t="n">
-        <v>0</v>
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>PAGO AL RESTAURANTE</t>
+        </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="10" t="inlineStr">
-        <is>
-          <t>TU GANANCIA después de pagarle</t>
-        </is>
-      </c>
-      <c r="B48" s="11">
-        <f>B43-B47</f>
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Ganancia antes de pagarle al restaurante</t>
+        </is>
+      </c>
+      <c r="B48" s="8">
+        <f>B40-B41-(B35+B36)</f>
         <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>Tu margen después de pagarle</t>
-        </is>
-      </c>
-      <c r="B49" s="14">
-        <f>IF(B35&gt;0,B48/B35,0)</f>
-        <v/>
+          <t>% de esa ganancia que le ofreces al restaurante</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="n">
+        <v>0.3</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="4" t="inlineStr">
-        <is>
-          <t>Máximo que puedes pagar sin perder dinero</t>
-        </is>
-      </c>
-      <c r="B50" s="8">
-        <f>MAX(0,B43)</f>
+      <c r="A50" s="10" t="inlineStr">
+        <is>
+          <t>PAGO SUGERIDO (redondeado a $5.000)</t>
+        </is>
+      </c>
+      <c r="B50" s="11">
+        <f>MAX(0,ROUNDDOWN(B48*B49/5000,0)*5000)</f>
         <v/>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>Aviso</t>
-        </is>
-      </c>
-      <c r="B51" s="13">
-        <f>IF(B47&gt;B43,"Cuidado: con ese pago pierdes dinero",IF(B49&lt;B8,"Ganas, pero por debajo de tu margen","Cumples tu margen"))</f>
-        <v/>
+          <t>…por persona</t>
+        </is>
+      </c>
+      <c r="B51" s="8">
+        <f>B50/B6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="10" t="inlineStr">
+        <is>
+          <t>LO QUE ACUERDAS PAGAR (escribe aquí; presupuesto de Sara: $500.000)</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="n">
+        <v>500000</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="3" t="inlineStr">
-        <is>
-          <t>CUÁNTO DEBE VALER EL CUPO</t>
-        </is>
+      <c r="A53" s="10" t="inlineStr">
+        <is>
+          <t>TU GANANCIA después de pagarle</t>
+        </is>
+      </c>
+      <c r="B53" s="11">
+        <f>B48-B52</f>
+        <v/>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>Precio mínimo (no pierdes ni ganas)</t>
-        </is>
-      </c>
-      <c r="B54" s="8">
-        <f>B33/(B6*(1-B9))</f>
+          <t>Tu margen después de pagarle</t>
+        </is>
+      </c>
+      <c r="B54" s="14">
+        <f>IF(B40&gt;0,B53/B40,0)</f>
         <v/>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="10" t="inlineStr">
-        <is>
-          <t>PRECIO RECOMENDADO para tu margen (redondeado a $5.000)</t>
-        </is>
-      </c>
-      <c r="B55" s="15">
-        <f>IF(1-B9-B8&lt;=0,"Revisa el margen",ROUNDUP(B33/(B6*(1-B9-B8))/5000,0)*5000)</f>
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Máximo que puedes pagar sin perder dinero</t>
+        </is>
+      </c>
+      <c r="B55" s="8">
+        <f>MAX(0,B48)</f>
         <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>Diferencia con el precio que cobras hoy</t>
-        </is>
-      </c>
-      <c r="B56" s="8">
-        <f>IF(ISNUMBER(B55),B55-B7,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="4" t="inlineStr">
-        <is>
-          <t>Máximo que puedes pagarle al lugar y mantener tu margen</t>
-        </is>
-      </c>
-      <c r="B57" s="8">
-        <f>B35*(1-B9-B8)-(B30+B31)</f>
-        <v/>
-      </c>
-      <c r="C57" s="2" t="inlineStr">
-        <is>
-          <t>(negativo = el precio no alcanza)</t>
+          <t>Aviso</t>
+        </is>
+      </c>
+      <c r="B56" s="13">
+        <f>IF(B52&gt;B48,"Cuidado: con ese pago pierdes dinero",IF(B54&lt;B8,"Ganas, pero por debajo de tu margen","Cumples tu margen"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>CUÁNTO DEBE VALER EL CUPO</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="3" t="inlineStr">
-        <is>
-          <t>PUNTO DE EQUILIBRIO</t>
-        </is>
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>Precio mínimo (no pierdes ni ganas)</t>
+        </is>
+      </c>
+      <c r="B59" s="8">
+        <f>B38/(B6*(1-B9))</f>
+        <v/>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="10" t="inlineStr">
         <is>
-          <t>Personas necesarias para no perder</t>
-        </is>
-      </c>
-      <c r="B60" s="16">
-        <f>IF(B7*(1-B9)-B28*(1+B10)&gt;0,ROUNDUP((B29*(1+B10)+B24)/(B7*(1-B9)-B28*(1+B10)),0),"No alcanza con este precio")</f>
+          <t>PRECIO RECOMENDADO para tu margen (redondeado a $5.000)</t>
+        </is>
+      </c>
+      <c r="B60" s="15">
+        <f>IF(1-B9-B8&lt;=0,"Revisa el margen",ROUNDUP(B38/(B6*(1-B9-B8))/5000,0)*5000)</f>
         <v/>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>Ingresos necesarios para no perder</t>
+          <t>Diferencia con el precio que cobras hoy</t>
         </is>
       </c>
       <c r="B61" s="8">
-        <f>IF(ISNUMBER(B60),B60*B7,"")</f>
+        <f>IF(ISNUMBER(B60),B60-B7,"")</f>
         <v/>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
+          <t>Máximo que puedes pagarle al restaurante y mantener tu margen</t>
+        </is>
+      </c>
+      <c r="B62" s="8">
+        <f>B40*(1-B9-B8)-(B35+B36)</f>
+        <v/>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>(negativo = el precio no alcanza)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>PUNTO DE EQUILIBRIO (aproximado: la pintura se compra en kits de 6 frascos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="10" t="inlineStr">
+        <is>
+          <t>Personas necesarias para no perder</t>
+        </is>
+      </c>
+      <c r="B65" s="16">
+        <f>IF(B7*(1-B9)-(B32+B14/B15)*(1+B10)&gt;0,ROUNDUP((B34*(1+B10)+B27)/(B7*(1-B9)-(B32+B14/B15)*(1+B10)),0),"No alcanza con este precio")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>Ingresos necesarios para no perder</t>
+        </is>
+      </c>
+      <c r="B66" s="8">
+        <f>IF(ISNUMBER(B65),B65*B7,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
           <t>Aporte de cada cupo a los costos fijos (precio menos su costo variable)</t>
         </is>
       </c>
-      <c r="B62" s="8">
-        <f>B7*(1-B9)-B28*(1+B10)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="4" t="inlineStr">
+      <c r="B67" s="8">
+        <f>B7*(1-B9)-(B32+B14/B15)*(1+B10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
         <is>
           <t>Personas por encima (+) o por debajo (−) del equilibrio</t>
         </is>
       </c>
-      <c r="B63" s="9">
-        <f>IF(ISNUMBER(B60),B6-B60,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="4" t="inlineStr">
+      <c r="B68" s="9">
+        <f>IF(ISNUMBER(B65),B6-B65,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
         <is>
           <t>¿Con tu número de personas cubres costos?</t>
         </is>
       </c>
-      <c r="B64" s="13">
-        <f>IF(ISNUMBER(B60),IF(B6&gt;=B60,"Sí, cubres costos","No, pierdes dinero"),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="3" t="inlineStr">
+      <c r="B69" s="13">
+        <f>IF(ISNUMBER(B65),IF(B6&gt;=B65,"Sí, cubres costos","No, pierdes dinero"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
         <is>
           <t>PRECIO DEL CUPO SEGÚN EL MARGEN QUE QUIERAS</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="17" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="17" t="inlineStr">
         <is>
           <t>Margen</t>
         </is>
       </c>
-      <c r="B67" s="17" t="inlineStr">
+      <c r="B72" s="17" t="inlineStr">
         <is>
           <t>Precio del cupo</t>
         </is>
       </c>
-      <c r="C67" s="17" t="inlineStr">
+      <c r="C72" s="17" t="inlineStr">
         <is>
           <t>Ganancia total</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="18" t="n">
+    <row r="73">
+      <c r="A73" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="B68" s="8">
-        <f>IF(1-$B$9-A68&lt;=0,"",ROUNDUP($B$33/($B$6*(1-$B$9-A68))/5000,0)*5000)</f>
-        <v/>
-      </c>
-      <c r="C68" s="8">
-        <f>IF(ISNUMBER(B68),B68*$B$6*(1-$B$9)-$B$33,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="18" t="n">
+      <c r="B73" s="8">
+        <f>IF(1-B9-A73&lt;=0,"",ROUNDUP(B38/(B6*(1-B9-A73))/5000,0)*5000)</f>
+        <v/>
+      </c>
+      <c r="C73" s="8">
+        <f>IF(ISNUMBER(B73),B73*B6*(1-B9)-B38,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="18" t="n">
         <v>0.3</v>
       </c>
-      <c r="B69" s="8">
-        <f>IF(1-$B$9-A69&lt;=0,"",ROUNDUP($B$33/($B$6*(1-$B$9-A69))/5000,0)*5000)</f>
-        <v/>
-      </c>
-      <c r="C69" s="8">
-        <f>IF(ISNUMBER(B69),B69*$B$6*(1-$B$9)-$B$33,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="18" t="n">
+      <c r="B74" s="8">
+        <f>IF(1-B9-A74&lt;=0,"",ROUNDUP(B38/(B6*(1-B9-A74))/5000,0)*5000)</f>
+        <v/>
+      </c>
+      <c r="C74" s="8">
+        <f>IF(ISNUMBER(B74),B74*B6*(1-B9)-B38,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="18" t="n">
         <v>0.4</v>
       </c>
-      <c r="B70" s="8">
-        <f>IF(1-$B$9-A70&lt;=0,"",ROUNDUP($B$33/($B$6*(1-$B$9-A70))/5000,0)*5000)</f>
-        <v/>
-      </c>
-      <c r="C70" s="8">
-        <f>IF(ISNUMBER(B70),B70*$B$6*(1-$B$9)-$B$33,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="18" t="n">
+      <c r="B75" s="8">
+        <f>IF(1-B9-A75&lt;=0,"",ROUNDUP(B38/(B6*(1-B9-A75))/5000,0)*5000)</f>
+        <v/>
+      </c>
+      <c r="C75" s="8">
+        <f>IF(ISNUMBER(B75),B75*B6*(1-B9)-B38,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="18" t="n">
         <v>0.5</v>
       </c>
-      <c r="B71" s="8">
-        <f>IF(1-$B$9-A71&lt;=0,"",ROUNDUP($B$33/($B$6*(1-$B$9-A71))/5000,0)*5000)</f>
-        <v/>
-      </c>
-      <c r="C71" s="8">
-        <f>IF(ISNUMBER(B71),B71*$B$6*(1-$B$9)-$B$33,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="3" t="inlineStr">
+      <c r="B76" s="8">
+        <f>IF(1-B9-A76&lt;=0,"",ROUNDUP(B38/(B6*(1-B9-A76))/5000,0)*5000)</f>
+        <v/>
+      </c>
+      <c r="C76" s="8">
+        <f>IF(ISNUMBER(B76),B76*B6*(1-B9)-B38,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
         <is>
           <t>SI CAMBIA EL NÚMERO DE PERSONAS</t>
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" s="17" t="inlineStr">
+    <row r="79">
+      <c r="A79" s="17" t="inlineStr">
         <is>
           <t>Personas</t>
         </is>
       </c>
-      <c r="B74" s="17" t="inlineStr">
+      <c r="B79" s="17" t="inlineStr">
         <is>
           <t>Ingresos</t>
         </is>
       </c>
-      <c r="C74" s="17" t="inlineStr">
+      <c r="C79" s="17" t="inlineStr">
         <is>
           <t>Costo total</t>
         </is>
       </c>
-      <c r="D74" s="17" t="inlineStr">
+      <c r="D79" s="17" t="inlineStr">
         <is>
           <t>Ganancia</t>
         </is>
       </c>
-      <c r="E74" s="17" t="inlineStr">
+      <c r="E79" s="17" t="inlineStr">
         <is>
           <t>Margen</t>
         </is>
       </c>
-      <c r="F74" s="17" t="inlineStr">
+      <c r="F79" s="17" t="inlineStr">
         <is>
           <t>Precio para tu margen</t>
         </is>
       </c>
-      <c r="G74" s="17" t="inlineStr">
+      <c r="G79" s="17" t="inlineStr">
         <is>
           <t>¿Cubre costos?</t>
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="19" t="n">
-        <v>6</v>
-      </c>
-      <c r="B75" s="8">
-        <f>$B$7*A75</f>
-        <v/>
-      </c>
-      <c r="C75" s="8">
-        <f>($B$29+$B$28*A75)*(1+$B$10)+$B$24</f>
-        <v/>
-      </c>
-      <c r="D75" s="20">
-        <f>B75*(1-$B$9)-C75</f>
-        <v/>
-      </c>
-      <c r="E75" s="14">
-        <f>IF(B75&gt;0,D75/B75,0)</f>
-        <v/>
-      </c>
-      <c r="F75" s="8">
-        <f>IF(1-$B$9-$B$8&lt;=0,"",ROUNDUP(C75/(A75*(1-$B$9-$B$8))/5000,0)*5000)</f>
-        <v/>
-      </c>
-      <c r="G75" s="13">
-        <f>IF(D75&gt;=0,"Sí","No: pierdes")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="19" t="n">
+    <row r="80">
+      <c r="A80" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="B76" s="8">
-        <f>$B$7*A76</f>
-        <v/>
-      </c>
-      <c r="C76" s="8">
-        <f>($B$29+$B$28*A76)*(1+$B$10)+$B$24</f>
-        <v/>
-      </c>
-      <c r="D76" s="20">
-        <f>B76*(1-$B$9)-C76</f>
-        <v/>
-      </c>
-      <c r="E76" s="14">
-        <f>IF(B76&gt;0,D76/B76,0)</f>
-        <v/>
-      </c>
-      <c r="F76" s="8">
-        <f>IF(1-$B$9-$B$8&lt;=0,"",ROUNDUP(C76/(A76*(1-$B$9-$B$8))/5000,0)*5000)</f>
-        <v/>
-      </c>
-      <c r="G76" s="13">
-        <f>IF(D76&gt;=0,"Sí","No: pierdes")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="19" t="n">
+      <c r="B80" s="8">
+        <f>B7*A80</f>
+        <v/>
+      </c>
+      <c r="C80" s="8">
+        <f>(B34+B32*A80+ROUNDUP(A80/B15,0)*B14)*(1+B10)+B27</f>
+        <v/>
+      </c>
+      <c r="D80" s="20">
+        <f>B80*(1-B9)-C80</f>
+        <v/>
+      </c>
+      <c r="E80" s="14">
+        <f>IF(B80&gt;0,D80/B80,0)</f>
+        <v/>
+      </c>
+      <c r="F80" s="8">
+        <f>IF(1-B9-B8&lt;=0,"",ROUNDUP(C80/(A80*(1-B9-B8))/5000,0)*5000)</f>
+        <v/>
+      </c>
+      <c r="G80" s="13">
+        <f>IF(D80&gt;=0,"Sí","No: pierdes")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="B77" s="8">
-        <f>$B$7*A77</f>
-        <v/>
-      </c>
-      <c r="C77" s="8">
-        <f>($B$29+$B$28*A77)*(1+$B$10)+$B$24</f>
-        <v/>
-      </c>
-      <c r="D77" s="20">
-        <f>B77*(1-$B$9)-C77</f>
-        <v/>
-      </c>
-      <c r="E77" s="14">
-        <f>IF(B77&gt;0,D77/B77,0)</f>
-        <v/>
-      </c>
-      <c r="F77" s="8">
-        <f>IF(1-$B$9-$B$8&lt;=0,"",ROUNDUP(C77/(A77*(1-$B$9-$B$8))/5000,0)*5000)</f>
-        <v/>
-      </c>
-      <c r="G77" s="13">
-        <f>IF(D77&gt;=0,"Sí","No: pierdes")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="19" t="n">
-        <v>11</v>
-      </c>
-      <c r="B78" s="8">
-        <f>$B$7*A78</f>
-        <v/>
-      </c>
-      <c r="C78" s="8">
-        <f>($B$29+$B$28*A78)*(1+$B$10)+$B$24</f>
-        <v/>
-      </c>
-      <c r="D78" s="20">
-        <f>B78*(1-$B$9)-C78</f>
-        <v/>
-      </c>
-      <c r="E78" s="14">
-        <f>IF(B78&gt;0,D78/B78,0)</f>
-        <v/>
-      </c>
-      <c r="F78" s="8">
-        <f>IF(1-$B$9-$B$8&lt;=0,"",ROUNDUP(C78/(A78*(1-$B$9-$B$8))/5000,0)*5000)</f>
-        <v/>
-      </c>
-      <c r="G78" s="13">
-        <f>IF(D78&gt;=0,"Sí","No: pierdes")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="19" t="n">
+      <c r="B81" s="8">
+        <f>B7*A81</f>
+        <v/>
+      </c>
+      <c r="C81" s="8">
+        <f>(B34+B32*A81+ROUNDUP(A81/B15,0)*B14)*(1+B10)+B27</f>
+        <v/>
+      </c>
+      <c r="D81" s="20">
+        <f>B81*(1-B9)-C81</f>
+        <v/>
+      </c>
+      <c r="E81" s="14">
+        <f>IF(B81&gt;0,D81/B81,0)</f>
+        <v/>
+      </c>
+      <c r="F81" s="8">
+        <f>IF(1-B9-B8&lt;=0,"",ROUNDUP(C81/(A81*(1-B9-B8))/5000,0)*5000)</f>
+        <v/>
+      </c>
+      <c r="G81" s="13">
+        <f>IF(D81&gt;=0,"Sí","No: pierdes")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="19" t="n">
         <v>12</v>
       </c>
-      <c r="B79" s="8">
-        <f>$B$7*A79</f>
-        <v/>
-      </c>
-      <c r="C79" s="8">
-        <f>($B$29+$B$28*A79)*(1+$B$10)+$B$24</f>
-        <v/>
-      </c>
-      <c r="D79" s="20">
-        <f>B79*(1-$B$9)-C79</f>
-        <v/>
-      </c>
-      <c r="E79" s="14">
-        <f>IF(B79&gt;0,D79/B79,0)</f>
-        <v/>
-      </c>
-      <c r="F79" s="8">
-        <f>IF(1-$B$9-$B$8&lt;=0,"",ROUNDUP(C79/(A79*(1-$B$9-$B$8))/5000,0)*5000)</f>
-        <v/>
-      </c>
-      <c r="G79" s="13">
-        <f>IF(D79&gt;=0,"Sí","No: pierdes")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="2" t="inlineStr">
-        <is>
-          <t>Nota: las pinturas textiles necesitan fijarse con calor (plancha o vapor) después de pintar; si se hace en el taller, hay que prever la plancha.</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="2" t="inlineStr">
-        <is>
-          <t>Los datos marcados ESTIMADO no son cotizaciones reales. El pago al lugar se descuenta de tu ganancia y los escenarios lo usan.</t>
+      <c r="B82" s="8">
+        <f>B7*A82</f>
+        <v/>
+      </c>
+      <c r="C82" s="8">
+        <f>(B34+B32*A82+ROUNDUP(A82/B15,0)*B14)*(1+B10)+B27</f>
+        <v/>
+      </c>
+      <c r="D82" s="20">
+        <f>B82*(1-B9)-C82</f>
+        <v/>
+      </c>
+      <c r="E82" s="14">
+        <f>IF(B82&gt;0,D82/B82,0)</f>
+        <v/>
+      </c>
+      <c r="F82" s="8">
+        <f>IF(1-B9-B8&lt;=0,"",ROUNDUP(C82/(A82*(1-B9-B8))/5000,0)*5000)</f>
+        <v/>
+      </c>
+      <c r="G82" s="13">
+        <f>IF(D82&gt;=0,"Sí","No: pierdes")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="B83" s="8">
+        <f>B7*A83</f>
+        <v/>
+      </c>
+      <c r="C83" s="8">
+        <f>(B34+B32*A83+ROUNDUP(A83/B15,0)*B14)*(1+B10)+B27</f>
+        <v/>
+      </c>
+      <c r="D83" s="20">
+        <f>B83*(1-B9)-C83</f>
+        <v/>
+      </c>
+      <c r="E83" s="14">
+        <f>IF(B83&gt;0,D83/B83,0)</f>
+        <v/>
+      </c>
+      <c r="F83" s="8">
+        <f>IF(1-B9-B8&lt;=0,"",ROUNDUP(C83/(A83*(1-B9-B8))/5000,0)*5000)</f>
+        <v/>
+      </c>
+      <c r="G83" s="13">
+        <f>IF(D83&gt;=0,"Sí","No: pierdes")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B84" s="8">
+        <f>B7*A84</f>
+        <v/>
+      </c>
+      <c r="C84" s="8">
+        <f>(B34+B32*A84+ROUNDUP(A84/B15,0)*B14)*(1+B10)+B27</f>
+        <v/>
+      </c>
+      <c r="D84" s="20">
+        <f>B84*(1-B9)-C84</f>
+        <v/>
+      </c>
+      <c r="E84" s="14">
+        <f>IF(B84&gt;0,D84/B84,0)</f>
+        <v/>
+      </c>
+      <c r="F84" s="8">
+        <f>IF(1-B9-B8&lt;=0,"",ROUNDUP(C84/(A84*(1-B9-B8))/5000,0)*5000)</f>
+        <v/>
+      </c>
+      <c r="G84" s="13">
+        <f>IF(D84&gt;=0,"Sí","No: pierdes")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>Nota: las pinturas textiles se fijan con calor (plancha o vapor) después de pintar; hay que prever plancha y enchufes en el restaurante.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>Los datos marcados ESTIMADO no son cotizaciones reales. El pago al restaurante se descuenta de tu ganancia y los escenarios lo usan.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A66:G66"/>
+    <mergeCell ref="A58:G58"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A53:G53"/>
-    <mergeCell ref="A26:G26"/>
+    <mergeCell ref="A87:G87"/>
+    <mergeCell ref="A78:G78"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A42:G42"/>
-    <mergeCell ref="A59:G59"/>
-    <mergeCell ref="A81:G81"/>
-    <mergeCell ref="A73:G73"/>
-    <mergeCell ref="A82:G82"/>
+    <mergeCell ref="A86:G86"/>
+    <mergeCell ref="A29:G29"/>
+    <mergeCell ref="A64:G64"/>
+    <mergeCell ref="A71:G71"/>
+    <mergeCell ref="A47:G47"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Textile workshop quote: kimono cost 80k (confirmed)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FV7y6XEE3x9ogCMyfe3pnd
</commit_message>
<xml_diff>
--- a/docs/sesion-2026-10-02/cotizacion-taller-pintura-textil.xlsx
+++ b/docs/sesion-2026-10-02/cotizacion-taller-pintura-textil.xlsx
@@ -238,7 +238,7 @@
     </comment>
     <comment ref="B12" authorId="0" shapeId="0">
       <text>
-        <t>ESTIMADO Y PENDIENTE: Sara no alcanzó a enviar el costo real. Es el costo más importante.</t>
+        <t>Dato de Sara.</t>
       </text>
     </comment>
     <comment ref="B13" authorId="0" shapeId="0">
@@ -643,7 +643,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Edita solo las celdas AMARILLAS. Lo marcado ESTIMADO no es un dato real: reemplázalo, sobre todo el costo del kimono.</t>
+          <t>Edita solo las celdas AMARILLAS. Lo marcado ESTIMADO no es un dato real: reemplázalo cuando lo tengas.</t>
         </is>
       </c>
     </row>
@@ -721,7 +721,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>120000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="13">

</xml_diff>